<commit_message>
Add common-change analysis and full text review queue
</commit_message>
<xml_diff>
--- a/outputs/resultats/bnc/2026_t2_vs_2026_t1/comparison.xlsx
+++ b/outputs/resultats/bnc/2026_t2_vs_2026_t1/comparison.xlsx
@@ -585,16 +585,8 @@
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28T18:14:18.809065+00:00</t>
-        </is>
-      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -655,7 +647,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28T17:56:50.378371+00:00</t>
+          <t>2026-06-05T19:44:58.066138+00:00</t>
         </is>
       </c>
     </row>
@@ -718,7 +710,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28T17:56:28.464078+00:00</t>
+          <t>2026-06-05T19:39:30.795077+00:00</t>
         </is>
       </c>
     </row>
@@ -840,7 +832,7 @@
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-28T17:56:28.861267+00:00</t>
+          <t>2026-06-05T19:45:10.715516+00:00</t>
         </is>
       </c>
     </row>
@@ -935,8 +927,16 @@
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr"/>
-      <c r="L8" s="3" t="inlineStr"/>
-      <c r="M8" s="3" t="inlineStr"/>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05T19:45:08.896124+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -982,8 +982,16 @@
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr"/>
-      <c r="L9" s="3" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05T19:45:06.774270+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1080,8 +1088,16 @@
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr"/>
-      <c r="L11" s="3" t="inlineStr"/>
-      <c r="M11" s="3" t="inlineStr"/>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05T19:45:04.895920+00:00</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:M11"/>

</xml_diff>